<commit_message>
Import/Export forecast and stabilised v5
</commit_message>
<xml_diff>
--- a/app/templates/report/stabilised.xlsx
+++ b/app/templates/report/stabilised.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Development\projects\ciber\cotown\back\app\templates\report\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48ED91D5-6B62-4B85-98B8-9D8329D50C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C475D9A1-E1E7-4506-8FE2-D928F2BBE5D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="750" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,15 +69,6 @@
     <t>Occupancy</t>
   </si>
   <si>
-    <t>Rent_long</t>
-  </si>
-  <si>
-    <t>Rent_medium</t>
-  </si>
-  <si>
-    <t>Rent_short</t>
-  </si>
-  <si>
     <t>% Occup.</t>
   </si>
   <si>
@@ -86,6 +77,15 @@
   </si>
   <si>
     <t>Leakage</t>
+  </si>
+  <si>
+    <t>Pct_long</t>
+  </si>
+  <si>
+    <t>Pct_medium</t>
+  </si>
+  <si>
+    <t>Pct_short</t>
   </si>
 </sst>
 </file>
@@ -294,20 +294,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <font>
-        <strike val="0"/>
-      </font>
-      <border>
-        <top style="hair">
-          <color auto="1"/>
-        </top>
-        <bottom/>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <strike val="0"/>
@@ -721,7 +708,7 @@
         <v>0</v>
       </c>
       <c r="C1" s="12" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D1" s="12" t="s">
         <v>1</v>
@@ -736,7 +723,7 @@
         <v>4</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="14.25" x14ac:dyDescent="0.3">
@@ -750,17 +737,17 @@
         <v>8</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="E2" s="11" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="G2" s="14"/>
       <c r="H2" s="11" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -779,12 +766,7 @@
   </sheetData>
   <autoFilter ref="A1:G1" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="A3:G99999">
-    <cfRule type="expression" dxfId="1" priority="2">
-      <formula>$A2&gt;$A3</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H99999">
+  <conditionalFormatting sqref="A3:H99999">
     <cfRule type="expression" dxfId="0" priority="1">
       <formula>$A2&gt;$A3</formula>
     </cfRule>

</xml_diff>